<commit_message>
planilha atualizada - 27/08/2026 12:33 UTC (via repository_dispatch)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -29163,13 +29163,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6E98AE7-5A0C-4695-B93A-67B19F42BA1D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D0AB89C-C312-4E52-87D7-BD3E44131876}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1BF0E13-84BA-42B4-A056-8EA70F314F0D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5A8E3C4-7D46-44EA-963D-65E94663DB0F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93424EF1-901B-4B2E-87D9-822AA653BF4E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD2ECB1E-0A91-416F-B35F-09DD4FF313CF}"/>
 </file>
</xml_diff>